<commit_message>
chore(invoice): use new unified freelancer template; single 양식 다운로드 button; parse 은행계좌 label
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/public/freelancer-individual-template.xlsx
+++ b/app/public/freelancer-individual-template.xlsx
@@ -8,29 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juliekim/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{90A5D637-CC1A-2D4D-9455-8CE6DBA76E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{283175AF-D9C5-8846-94E6-F33C4A937295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Korean" sheetId="1" r:id="rId1"/>
+    <sheet name="English" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
   <si>
     <t>No.</t>
   </si>
   <si>
-    <t>견적서</t>
-  </si>
-  <si>
-    <t>날 짜</t>
-  </si>
-  <si>
     <t>공급자 / 프리랜서</t>
   </si>
   <si>
@@ -70,279 +65,108 @@
     <t>비고</t>
   </si>
   <si>
-    <t>합 계</t>
+    <t xml:space="preserve">날 짜 </t>
+  </si>
+  <si>
+    <t>Invoice</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Date</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>Upload Date</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>Freelancer Information</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>ID number</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>Name</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone </t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>Email</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>Video Title</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>Unit Price</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>Total</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>Remark</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>To</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>Invoice details as below.</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">BANK Account Information : </t>
+    <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
     <r>
       <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Malgun Gothic"/>
         <family val="2"/>
         <charset val="129"/>
       </rPr>
-      <t>입금계좌</t>
+      <t>은행계좌</t>
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정보</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> : </t>
     </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t>토스뱅크</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> 1000-2534-2158</t>
-    </r>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>05.01 CDS 비교분석</t>
-  </si>
-  <si>
-    <t>05.01 편입</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>05.04 debate</t>
-  </si>
-  <si>
-    <t>05.04 진로탐색</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">05.05 fit </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>대학교</t>
-    </r>
-  </si>
-  <si>
-    <t>05.07 2. 왜 미국 대학은 ‘수상 개수’보다 ‘수상의 맥락’을 더 중요하게 볼까</t>
-  </si>
-  <si>
-    <t>05.08 공대 과목 선택</t>
-  </si>
-  <si>
-    <t>05.08 바이오 과목 선택</t>
-  </si>
-  <si>
-    <t>05.14 로드맵</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">05.14 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>홍보영상</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>05.15 (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>홍보영상</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) 04  Video #4  ·  Authentic Narrative</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>05.15 (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>홍보영상</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">) 05 Video #5  ·  Final CTA  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>희소성</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>모집</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">05.19 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>논현동</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">05.19 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>톡</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>논현동</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">05.22 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>공대</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">05.22 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>디자인</t>
-    </r>
-  </si>
-  <si>
-    <t>홍보영상</t>
-    <phoneticPr fontId="7" type="noConversion"/>
+    <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -364,13 +188,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -414,20 +231,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="129"/>
-    </font>
-    <font>
       <u/>
       <sz val="10"/>
       <color theme="10"/>
@@ -444,17 +247,38 @@
       <charset val="129"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Malgun Gothic"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Arial"/>
-      <family val="3"/>
+      <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
+      <name val="Malgun Gothic"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
     </font>
@@ -809,9 +633,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -819,14 +643,14 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -857,48 +681,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -906,13 +709,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -938,6 +741,36 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1181,27 +1014,27 @@
       <c r="I1" s="3"/>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A2" s="32" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
+      <c r="A2" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
       <c r="I2" s="3"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A3" s="33"/>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
+      <c r="A3" s="26"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
       <c r="I3" s="3"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1">
@@ -1215,36 +1048,36 @@
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
     </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1">
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" thickTop="1">
       <c r="A5" s="3"/>
       <c r="B5" s="4" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C5" s="24"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="34" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="35"/>
-      <c r="G5" s="35"/>
-      <c r="H5" s="36"/>
+      <c r="E5" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="29"/>
       <c r="I5" s="3"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F6" s="20"/>
       <c r="G6" s="8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H6" s="23"/>
       <c r="I6" s="3"/>
@@ -1255,26 +1088,26 @@
       <c r="C7" s="9"/>
       <c r="D7" s="3"/>
       <c r="E7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="38"/>
+        <v>6</v>
+      </c>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="31"/>
       <c r="I7" s="3"/>
     </row>
     <row r="8" spans="1:9" ht="15.75" customHeight="1" thickBot="1">
       <c r="A8" s="3"/>
-      <c r="B8" s="39" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="33"/>
+      <c r="B8" s="32" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="26"/>
       <c r="D8" s="3"/>
       <c r="E8" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="40"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="42"/>
+        <v>8</v>
+      </c>
+      <c r="F8" s="33"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="35"/>
       <c r="I8" s="3"/>
     </row>
     <row r="9" spans="1:9" ht="15.75" customHeight="1" thickTop="1">
@@ -1305,113 +1138,73 @@
         <v>0</v>
       </c>
       <c r="C11" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="F11" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="G11" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="F11" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="G11" s="43" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="36"/>
+      <c r="H11" s="29"/>
       <c r="I11" s="3"/>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1">
       <c r="A12" s="13"/>
-      <c r="B12" s="16">
-        <v>1</v>
-      </c>
-      <c r="C12" s="7">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="D12" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="17"/>
       <c r="F12" s="17"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="45"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="38"/>
       <c r="I12" s="3"/>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1">
       <c r="A13" s="13"/>
-      <c r="B13" s="16">
-        <v>2</v>
-      </c>
-      <c r="C13" s="7">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B13" s="16"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="17"/>
       <c r="F13" s="17"/>
-      <c r="G13" s="44"/>
-      <c r="H13" s="45"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="38"/>
       <c r="I13" s="3"/>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1">
       <c r="A14" s="13"/>
-      <c r="B14" s="16">
-        <v>3</v>
-      </c>
-      <c r="C14" s="7">
-        <v>5.4</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B14" s="16"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="17"/>
       <c r="F14" s="17"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="45"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="38"/>
       <c r="I14" s="3"/>
     </row>
     <row r="15" spans="1:9" ht="15.75" customHeight="1">
       <c r="A15" s="13"/>
-      <c r="B15" s="16">
-        <v>4</v>
-      </c>
-      <c r="C15" s="7">
-        <v>5.4</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="E15" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="17"/>
-      <c r="G15" s="44"/>
-      <c r="H15" s="45"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="38"/>
       <c r="I15" s="3"/>
     </row>
     <row r="16" spans="1:9" ht="15.75" customHeight="1">
       <c r="A16" s="13"/>
-      <c r="B16" s="16">
-        <v>5</v>
-      </c>
-      <c r="C16" s="7">
-        <v>5.5</v>
-      </c>
-      <c r="D16" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="E16" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B16" s="16"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="17"/>
       <c r="G16" s="10"/>
       <c r="H16" s="19"/>
@@ -1419,18 +1212,10 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1">
       <c r="A17" s="13"/>
-      <c r="B17" s="16">
-        <v>6</v>
-      </c>
-      <c r="C17" s="7">
-        <v>5.7</v>
-      </c>
-      <c r="D17" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="17"/>
       <c r="G17" s="10"/>
       <c r="H17" s="19"/>
@@ -1438,18 +1223,10 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1">
       <c r="A18" s="13"/>
-      <c r="B18" s="16">
-        <v>7</v>
-      </c>
-      <c r="C18" s="7">
-        <v>5.8</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B18" s="16"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="17"/>
       <c r="F18" s="17"/>
       <c r="G18" s="10"/>
       <c r="H18" s="19"/>
@@ -1457,18 +1234,10 @@
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1">
       <c r="A19" s="13"/>
-      <c r="B19" s="16">
-        <v>8</v>
-      </c>
-      <c r="C19" s="7">
-        <v>5.8</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="E19" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B19" s="16"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="17"/>
       <c r="F19" s="17"/>
       <c r="G19" s="10"/>
       <c r="H19" s="19"/>
@@ -1476,18 +1245,10 @@
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1">
       <c r="A20" s="13"/>
-      <c r="B20" s="16">
-        <v>9</v>
-      </c>
-      <c r="C20" s="7">
-        <v>5.14</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="E20" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B20" s="16"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="17"/>
       <c r="F20" s="17"/>
       <c r="G20" s="10"/>
       <c r="H20" s="19"/>
@@ -1495,81 +1256,43 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1">
       <c r="A21" s="13"/>
-      <c r="B21" s="16">
-        <v>10</v>
-      </c>
-      <c r="C21" s="7">
-        <v>5.14</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="E21" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="17"/>
       <c r="F21" s="17"/>
-      <c r="G21" s="25" t="s">
-        <v>34</v>
-      </c>
+      <c r="G21" s="25"/>
       <c r="H21" s="19"/>
       <c r="I21" s="3"/>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1">
       <c r="A22" s="13"/>
-      <c r="B22" s="16">
-        <v>11</v>
-      </c>
-      <c r="C22" s="7">
-        <v>5.15</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="E22" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B22" s="16"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="17"/>
       <c r="F22" s="17"/>
-      <c r="G22" s="25" t="s">
-        <v>34</v>
-      </c>
+      <c r="G22" s="25"/>
       <c r="H22" s="19"/>
       <c r="I22" s="3"/>
     </row>
     <row r="23" spans="1:9" ht="15.75" customHeight="1">
       <c r="A23" s="13"/>
-      <c r="B23" s="16">
-        <v>12</v>
-      </c>
-      <c r="C23" s="7">
-        <v>5.15</v>
-      </c>
-      <c r="D23" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="E23" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B23" s="16"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="17"/>
-      <c r="G23" s="25" t="s">
-        <v>34</v>
-      </c>
+      <c r="G23" s="25"/>
       <c r="H23" s="19"/>
       <c r="I23" s="3"/>
     </row>
     <row r="24" spans="1:9" ht="15.75" customHeight="1">
       <c r="A24" s="13"/>
-      <c r="B24" s="16">
-        <v>13</v>
-      </c>
-      <c r="C24" s="7">
-        <v>5.19</v>
-      </c>
-      <c r="D24" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="E24" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B24" s="16"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="17"/>
       <c r="G24" s="10"/>
       <c r="H24" s="19"/>
@@ -1577,18 +1300,10 @@
     </row>
     <row r="25" spans="1:9" ht="15.75" customHeight="1">
       <c r="A25" s="13"/>
-      <c r="B25" s="16">
-        <v>14</v>
-      </c>
-      <c r="C25" s="7">
-        <v>5.19</v>
-      </c>
-      <c r="D25" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="E25" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B25" s="16"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="17"/>
       <c r="F25" s="17"/>
       <c r="G25" s="10"/>
       <c r="H25" s="19"/>
@@ -1596,18 +1311,10 @@
     </row>
     <row r="26" spans="1:9" ht="15.75" customHeight="1">
       <c r="A26" s="13"/>
-      <c r="B26" s="16">
-        <v>15</v>
-      </c>
-      <c r="C26" s="7">
-        <v>5.22</v>
-      </c>
-      <c r="D26" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="E26" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B26" s="16"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="17"/>
       <c r="F26" s="17"/>
       <c r="G26" s="10"/>
       <c r="H26" s="19"/>
@@ -1615,60 +1322,48 @@
     </row>
     <row r="27" spans="1:9" ht="15.75" customHeight="1">
       <c r="A27" s="13"/>
-      <c r="B27" s="16">
-        <v>16</v>
-      </c>
-      <c r="C27" s="7">
-        <v>5.22</v>
-      </c>
-      <c r="D27" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="E27" s="17">
-        <v>30000</v>
-      </c>
+      <c r="B27" s="16"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="17"/>
       <c r="F27" s="17"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="45"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="38"/>
       <c r="I27" s="3"/>
     </row>
     <row r="28" spans="1:9" ht="15.75" customHeight="1" thickBot="1">
       <c r="A28" s="13"/>
-      <c r="B28" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="C28" s="47"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="18">
-        <v>480000</v>
-      </c>
-      <c r="G28" s="49"/>
-      <c r="H28" s="50"/>
+      <c r="B28" s="39"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
+      <c r="E28" s="41"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="43"/>
       <c r="I28" s="3"/>
     </row>
     <row r="29" spans="1:9" ht="15.75" customHeight="1" thickTop="1">
       <c r="A29" s="3"/>
-      <c r="B29" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="28"/>
+      <c r="B29" s="53" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="48"/>
+      <c r="D29" s="48"/>
+      <c r="E29" s="48"/>
+      <c r="F29" s="48"/>
+      <c r="G29" s="48"/>
+      <c r="H29" s="49"/>
       <c r="I29" s="3"/>
     </row>
     <row r="30" spans="1:9" ht="15.75" customHeight="1" thickBot="1">
       <c r="A30" s="3"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="30"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="31"/>
+      <c r="B30" s="50"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="51"/>
+      <c r="H30" s="52"/>
       <c r="I30" s="3"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" customHeight="1" thickTop="1">
@@ -1710,7 +1405,431 @@
     <mergeCell ref="B28:E28"/>
     <mergeCell ref="G28:H28"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB23E13-519F-0E49-927B-E8372BC9B2C6}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:I32"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="4" max="4" width="86.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A2" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A3" s="26"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:9" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" thickTop="1">
+      <c r="A5" s="3"/>
+      <c r="B5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="24"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="20"/>
+      <c r="G6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="23"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A8" s="3"/>
+      <c r="B8" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="26"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="33"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" thickTop="1">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A10" s="3"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.75" customHeight="1" thickTop="1">
+      <c r="A11" s="13"/>
+      <c r="B11" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="45" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" s="29"/>
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A12" s="13"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A13" s="13"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="3"/>
+    </row>
+    <row r="14" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A14" s="13"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="15" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A15" s="13"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="38"/>
+      <c r="I15" s="3"/>
+    </row>
+    <row r="16" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A16" s="13"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="3"/>
+    </row>
+    <row r="17" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A17" s="13"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="3"/>
+    </row>
+    <row r="18" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A18" s="13"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="3"/>
+    </row>
+    <row r="19" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A19" s="13"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="3"/>
+    </row>
+    <row r="20" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A20" s="13"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="3"/>
+    </row>
+    <row r="21" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A21" s="13"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A22" s="13"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="3"/>
+    </row>
+    <row r="23" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A23" s="13"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="3"/>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A24" s="13"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="3"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A25" s="13"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="3"/>
+    </row>
+    <row r="26" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A26" s="13"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="3"/>
+    </row>
+    <row r="27" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A27" s="13"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="3"/>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A28" s="13"/>
+      <c r="B28" s="39"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
+      <c r="E28" s="41"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="43"/>
+      <c r="I28" s="3"/>
+    </row>
+    <row r="29" spans="1:9" ht="15.75" customHeight="1" thickTop="1">
+      <c r="A29" s="3"/>
+      <c r="B29" s="47" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" s="48"/>
+      <c r="D29" s="48"/>
+      <c r="E29" s="48"/>
+      <c r="F29" s="48"/>
+      <c r="G29" s="48"/>
+      <c r="H29" s="49"/>
+      <c r="I29" s="3"/>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A30" s="3"/>
+      <c r="B30" s="50"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="51"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="3"/>
+    </row>
+    <row r="31" spans="1:9" ht="15.75" customHeight="1" thickTop="1">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="B29:H30"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="A2:H3"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="G11:H11"/>
+  </mergeCells>
+  <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>